<commit_message>
Version sin costos y ajuste de emisiones N2O
</commit_message>
<xml_diff>
--- a/Energy/A1_Inputs/A-I_Classifier_Modes_Demand.xlsx
+++ b/Energy/A1_Inputs/A-I_Classifier_Modes_Demand.xlsx
@@ -1836,8 +1836,8 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100B8F814574E960A4499025803604D4DF4" ma:contentTypeVersion="9" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="613b0908c48a25395136f5b5d1e9264a">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4b2ff61d-e0c4-454b-ba72-44cf85c32a41" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f5652efc65d8021725ff526b59607fd6" ns2:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B8F814574E960A4499025803604D4DF4" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="314e7041d7d1561dbe33e80becf1c782">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4b2ff61d-e0c4-454b-ba72-44cf85c32a41" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="84c838da6aa04a0f137f8b0aba02cfe1" ns2:_="">
     <xsd:import namespace="4b2ff61d-e0c4-454b-ba72-44cf85c32a41"/>
     <xsd:element name="properties">
       <xsd:complexType>
@@ -1915,8 +1915,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -2024,5 +2024,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24A6CD07-8CC8-4324-BF66-D5979349F68D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{52C81F54-7392-4496-B7D5-A66FE4FD9EE6}"/>
 </file>
</xml_diff>